<commit_message>
auto probe card stuff
</commit_message>
<xml_diff>
--- a/io_pair_inputs/Shorted_signals.xlsx
+++ b/io_pair_inputs/Shorted_signals.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liam.deacon\Desktop\Testing Mask Generator\io_pair_inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7F4DD40-FF1B-451C-840E-1E315140DBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D03807AD-8073-4AA7-AEF1-4630CC3757C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1714" uniqueCount="506">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1698" uniqueCount="505">
   <si>
     <t>Pad</t>
   </si>
@@ -1562,9 +1562,6 @@
   </si>
   <si>
     <t>I/O</t>
-  </si>
-  <si>
-    <t>INPUT0</t>
   </si>
   <si>
     <t>OUTPUTSPLIT</t>
@@ -4357,6 +4354,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4730,7 +4731,7 @@
         <v>10</v>
       </c>
       <c r="I5" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="J5">
         <f t="shared" si="0"/>
@@ -4760,7 +4761,7 @@
         <v>10</v>
       </c>
       <c r="I6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="J6">
         <f t="shared" si="0"/>
@@ -4840,7 +4841,7 @@
         <v>10</v>
       </c>
       <c r="I9" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="J9">
         <f t="shared" si="0"/>
@@ -4870,7 +4871,7 @@
         <v>10</v>
       </c>
       <c r="I10" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="J10">
         <f t="shared" si="0"/>
@@ -5027,7 +5028,7 @@
         <v>125</v>
       </c>
       <c r="I16" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.3">
@@ -5119,9 +5120,6 @@
       <c r="H20" t="s">
         <v>10</v>
       </c>
-      <c r="I20" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
@@ -5257,7 +5255,7 @@
         <v>125</v>
       </c>
       <c r="I26" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.3">
@@ -5394,7 +5392,7 @@
         <v>10</v>
       </c>
       <c r="I32" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="33" spans="2:9" x14ac:dyDescent="0.3">
@@ -5420,7 +5418,7 @@
         <v>10</v>
       </c>
       <c r="I33" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.3">
@@ -5513,7 +5511,7 @@
         <v>10</v>
       </c>
       <c r="I37" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="38" spans="2:9" x14ac:dyDescent="0.3">
@@ -5539,7 +5537,7 @@
         <v>10</v>
       </c>
       <c r="I38" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.3">
@@ -6278,7 +6276,7 @@
         <v>125</v>
       </c>
       <c r="I72" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="73" spans="2:9" x14ac:dyDescent="0.3">
@@ -6304,7 +6302,7 @@
         <v>125</v>
       </c>
       <c r="I73" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="74" spans="2:9" x14ac:dyDescent="0.3">
@@ -6371,9 +6369,6 @@
       <c r="H76" t="s">
         <v>10</v>
       </c>
-      <c r="I76" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="77" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
@@ -6397,9 +6392,6 @@
       <c r="H77" t="s">
         <v>10</v>
       </c>
-      <c r="I77" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="78" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
@@ -6423,9 +6415,6 @@
       <c r="H78" t="s">
         <v>10</v>
       </c>
-      <c r="I78" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
@@ -6450,7 +6439,7 @@
         <v>125</v>
       </c>
       <c r="I79" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="80" spans="2:9" x14ac:dyDescent="0.3">
@@ -6522,7 +6511,7 @@
         <v>125</v>
       </c>
       <c r="I82" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="83" spans="2:9" x14ac:dyDescent="0.3">
@@ -6547,9 +6536,6 @@
       <c r="H83" t="s">
         <v>10</v>
       </c>
-      <c r="I83" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
@@ -6573,9 +6559,6 @@
       <c r="H84" t="s">
         <v>10</v>
       </c>
-      <c r="I84" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
@@ -6750,9 +6733,6 @@
       <c r="H92" t="s">
         <v>10</v>
       </c>
-      <c r="I92" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
@@ -7179,7 +7159,7 @@
         <v>125</v>
       </c>
       <c r="I111" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="112" spans="2:9" x14ac:dyDescent="0.3">
@@ -7251,7 +7231,7 @@
         <v>125</v>
       </c>
       <c r="I114" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="115" spans="2:9" x14ac:dyDescent="0.3">
@@ -7297,9 +7277,6 @@
       <c r="H116" t="s">
         <v>10</v>
       </c>
-      <c r="I116" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="117" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
@@ -7324,7 +7301,7 @@
         <v>125</v>
       </c>
       <c r="I117" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="118" spans="2:9" x14ac:dyDescent="0.3">
@@ -7417,7 +7394,7 @@
         <v>125</v>
       </c>
       <c r="I121" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="122" spans="2:9" x14ac:dyDescent="0.3">
@@ -7550,7 +7527,7 @@
         <v>125</v>
       </c>
       <c r="I127" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="128" spans="2:9" x14ac:dyDescent="0.3">
@@ -8154,9 +8131,6 @@
       <c r="H155" t="s">
         <v>10</v>
       </c>
-      <c r="I155" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="156" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B156" t="s">
@@ -8204,7 +8178,7 @@
         <v>10</v>
       </c>
       <c r="I157" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="158" spans="2:9" x14ac:dyDescent="0.3">
@@ -8230,7 +8204,7 @@
         <v>10</v>
       </c>
       <c r="I158" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="159" spans="2:9" x14ac:dyDescent="0.3">
@@ -8256,7 +8230,7 @@
         <v>10</v>
       </c>
       <c r="I159" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="160" spans="2:9" x14ac:dyDescent="0.3">
@@ -8303,7 +8277,7 @@
         <v>10</v>
       </c>
       <c r="I161" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="162" spans="2:9" x14ac:dyDescent="0.3">
@@ -8573,9 +8547,6 @@
       <c r="H173" t="s">
         <v>10</v>
       </c>
-      <c r="I173" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="174" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B174" t="s">
@@ -8645,9 +8616,6 @@
       <c r="H176" t="s">
         <v>10</v>
       </c>
-      <c r="I176" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="177" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B177" t="s">
@@ -8716,7 +8684,7 @@
         <v>18</v>
       </c>
       <c r="I179" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="180" spans="2:9" x14ac:dyDescent="0.3">
@@ -8786,7 +8754,7 @@
         <v>18</v>
       </c>
       <c r="I182" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="183" spans="2:9" x14ac:dyDescent="0.3">
@@ -8811,9 +8779,6 @@
       <c r="H183" t="s">
         <v>10</v>
       </c>
-      <c r="I183" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="184" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B184" t="s">
@@ -8861,7 +8826,7 @@
         <v>10</v>
       </c>
       <c r="I185" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="186" spans="2:9" x14ac:dyDescent="0.3">
@@ -8887,7 +8852,7 @@
         <v>10</v>
       </c>
       <c r="I186" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="187" spans="2:9" x14ac:dyDescent="0.3">
@@ -8978,7 +8943,7 @@
         <v>10</v>
       </c>
       <c r="I190" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="191" spans="2:9" x14ac:dyDescent="0.3">
@@ -9004,7 +8969,7 @@
         <v>10</v>
       </c>
       <c r="I191" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="192" spans="2:9" x14ac:dyDescent="0.3">
@@ -9030,7 +8995,7 @@
         <v>18</v>
       </c>
       <c r="I192" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="193" spans="2:9" x14ac:dyDescent="0.3">
@@ -9055,9 +9020,6 @@
       <c r="H193" t="s">
         <v>10</v>
       </c>
-      <c r="I193" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="194" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B194" t="s">
@@ -9191,7 +9153,7 @@
         <v>125</v>
       </c>
       <c r="I199" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="200" spans="2:9" x14ac:dyDescent="0.3">
@@ -9281,9 +9243,6 @@
       <c r="H203" t="s">
         <v>10</v>
       </c>
-      <c r="I203" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="204" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B204" t="s">
@@ -9502,9 +9461,6 @@
       <c r="H213" t="s">
         <v>10</v>
       </c>
-      <c r="I213" t="s">
-        <v>501</v>
-      </c>
     </row>
     <row r="214" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B214" t="s">
@@ -9598,7 +9554,7 @@
         <v>125</v>
       </c>
       <c r="I217" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="218" spans="2:9" x14ac:dyDescent="0.3">
@@ -9624,7 +9580,7 @@
         <v>18</v>
       </c>
       <c r="I218" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="219" spans="2:9" x14ac:dyDescent="0.3">
@@ -9694,7 +9650,7 @@
         <v>125</v>
       </c>
       <c r="I221" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="222" spans="2:9" x14ac:dyDescent="0.3">
@@ -9762,7 +9718,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="225" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="225" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B225" t="s">
         <v>174</v>
       </c>
@@ -9785,7 +9741,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="226" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="226" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B226" t="s">
         <v>177</v>
       </c>
@@ -9806,7 +9762,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="227" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="227" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B227" t="s">
         <v>178</v>
       </c>
@@ -9828,11 +9784,8 @@
       <c r="H227" t="s">
         <v>10</v>
       </c>
-      <c r="I227" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="228" spans="2:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="228" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B228" t="s">
         <v>180</v>
       </c>
@@ -9853,7 +9806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="229" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="229" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B229" t="s">
         <v>21</v>
       </c>
@@ -9876,7 +9829,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="230" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="230" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B230" t="s">
         <v>24</v>
       </c>
@@ -9899,20 +9852,20 @@
         <v>10</v>
       </c>
     </row>
-    <row r="233" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="233" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B233" t="s">
         <v>464</v>
       </c>
       <c r="F233" s="1"/>
       <c r="G233" s="1"/>
     </row>
-    <row r="234" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="234" spans="2:8" x14ac:dyDescent="0.3">
       <c r="F234" t="s">
         <v>465</v>
       </c>
       <c r="G234" s="1"/>
     </row>
-    <row r="236" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="236" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B236" t="s">
         <v>466</v>
       </c>
@@ -9920,7 +9873,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="237" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="237" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B237" t="s">
         <v>468</v>
       </c>
@@ -14163,27 +14116,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <FinalVersion xmlns="fecdb0e0-fc7a-47f6-8975-a11fd98dcca7" xsi:nil="true"/>
-    <TaxCatchAll xmlns="33ec47e1-1855-4fdb-a465-ff807d380ac7" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fecdb0e0-fc7a-47f6-8975-a11fd98dcca7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010067901BB0E6A75C42A8307BAB3B98A585" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="06c3f6fbc4138a297af263222011e8d6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="fecdb0e0-fc7a-47f6-8975-a11fd98dcca7" xmlns:ns3="33ec47e1-1855-4fdb-a465-ff807d380ac7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d2fc8ffc4f33fb0612843664240ddc4d" ns2:_="" ns3:_="">
     <xsd:import namespace="fecdb0e0-fc7a-47f6-8975-a11fd98dcca7"/>
@@ -14452,10 +14384,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <FinalVersion xmlns="fecdb0e0-fc7a-47f6-8975-a11fd98dcca7" xsi:nil="true"/>
+    <TaxCatchAll xmlns="33ec47e1-1855-4fdb-a465-ff807d380ac7" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="fecdb0e0-fc7a-47f6-8975-a11fd98dcca7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{971EEB71-7CEF-4275-BE9C-3DD35F3C9DF0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C66F34F-E70E-45C7-A121-B069CD177291}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="fecdb0e0-fc7a-47f6-8975-a11fd98dcca7"/>
+    <ds:schemaRef ds:uri="33ec47e1-1855-4fdb-a465-ff807d380ac7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -14472,20 +14436,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C66F34F-E70E-45C7-A121-B069CD177291}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{971EEB71-7CEF-4275-BE9C-3DD35F3C9DF0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="fecdb0e0-fc7a-47f6-8975-a11fd98dcca7"/>
-    <ds:schemaRef ds:uri="33ec47e1-1855-4fdb-a465-ff807d380ac7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>